<commit_message>
Primera cosecha de cotizaciones RFQ vaciada al Excel y reprecio
24 cotizaciones reales de <24h (cotizaciones-rfq.md); 15 SKUs pasan a FOB [V-RFQ].
Oficina y exterior cotizaron 50-60% abajo del estimado (se bajan EQP-501/701 para
competir); madera y lounge arriba (suben EQP-102/105/301/401). Margen mínimo 35% sostenido.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/investigacion/EQUIPA-CATALOGO-MAESTRO.xlsx
+++ b/investigacion/EQUIPA-CATALOGO-MAESTRO.xlsx
@@ -957,7 +957,7 @@
         </is>
       </c>
       <c r="D2" s="14" t="n">
-        <v>26</v>
+        <v>17</v>
       </c>
       <c r="E2" s="15" t="n">
         <v>0.12</v>
@@ -1027,12 +1027,12 @@
       </c>
       <c r="V2" s="13" t="inlineStr">
         <is>
-          <t>[V]</t>
+          <t>[V-RFQ]</t>
         </is>
       </c>
       <c r="W2" s="22" t="inlineStr">
         <is>
-          <t>Tianjin Okay Int'l — tianjinokayfurniture.en.made-in-china.com (velvet metal $24-26 a 200+)</t>
+          <t>RFQ 20-ago: Tianjin NOKA $16.90 / Shijiazhuang Adxin $12 / Bazhou Xinju $26 (velvet metal)</t>
         </is>
       </c>
     </row>
@@ -1053,7 +1053,7 @@
         </is>
       </c>
       <c r="D3" s="14" t="n">
-        <v>30</v>
+        <v>38</v>
       </c>
       <c r="E3" s="15" t="n">
         <v>0.17</v>
@@ -1095,10 +1095,10 @@
         <v/>
       </c>
       <c r="O3" s="19" t="n">
-        <v>1890</v>
+        <v>2090</v>
       </c>
       <c r="P3" s="19" t="n">
-        <v>2290</v>
+        <v>2490</v>
       </c>
       <c r="Q3" s="20">
         <f>O3-N3</f>
@@ -1123,12 +1123,12 @@
       </c>
       <c r="V3" s="13" t="inlineStr">
         <is>
-          <t>[V]</t>
+          <t>[V-RFQ]</t>
         </is>
       </c>
       <c r="W3" s="22" t="inlineStr">
         <is>
-          <t>Qingdao Welhome — welhome.en.made-in-china.com (bentwood haya $25-38)</t>
+          <t>RFQ 20-ago: Ganzhou Nanyi $38 (nórdica madera maciza)</t>
         </is>
       </c>
     </row>
@@ -1245,7 +1245,7 @@
         </is>
       </c>
       <c r="D5" s="14" t="n">
-        <v>28</v>
+        <v>17</v>
       </c>
       <c r="E5" s="15" t="n">
         <v>0.12</v>
@@ -1315,12 +1315,12 @@
       </c>
       <c r="V5" s="13" t="inlineStr">
         <is>
-          <t>[V]</t>
+          <t>[V-RFQ]</t>
         </is>
       </c>
       <c r="W5" s="22" t="inlineStr">
         <is>
-          <t>Tianjin Okay / Zhuoguan $20.90-29.90 (made-in-china.com)</t>
+          <t>RFQ 20-ago: mismas cotizaciones sillas tapizadas ($12-26)</t>
         </is>
       </c>
     </row>
@@ -1341,7 +1341,7 @@
         </is>
       </c>
       <c r="D6" s="14" t="n">
-        <v>35</v>
+        <v>38</v>
       </c>
       <c r="E6" s="15" t="n">
         <v>0.17</v>
@@ -1383,10 +1383,10 @@
         <v/>
       </c>
       <c r="O6" s="19" t="n">
-        <v>1990</v>
+        <v>2090</v>
       </c>
       <c r="P6" s="19" t="n">
-        <v>2390</v>
+        <v>2490</v>
       </c>
       <c r="Q6" s="20">
         <f>O6-N6</f>
@@ -1411,12 +1411,12 @@
       </c>
       <c r="V6" s="13" t="inlineStr">
         <is>
-          <t>[E]</t>
+          <t>[V-RFQ]</t>
         </is>
       </c>
       <c r="W6" s="22" t="inlineStr">
         <is>
-          <t>Interpolado Welhome/CDG (madera+tapiz)</t>
+          <t>RFQ 20-ago: Ganzhou Nanyi $38</t>
         </is>
       </c>
     </row>
@@ -1437,7 +1437,7 @@
         </is>
       </c>
       <c r="D7" s="14" t="n">
-        <v>31</v>
+        <v>17</v>
       </c>
       <c r="E7" s="15" t="n">
         <v>0.13</v>
@@ -1507,12 +1507,12 @@
       </c>
       <c r="V7" s="13" t="inlineStr">
         <is>
-          <t>[V]</t>
+          <t>[V-RFQ]</t>
         </is>
       </c>
       <c r="W7" s="22" t="inlineStr">
         <is>
-          <t>Alibaba showroom velvet dining chair $18-31.5</t>
+          <t>RFQ 20-ago: velvet $12-26 (NOKA/Adxin/Xinju)</t>
         </is>
       </c>
     </row>
@@ -1533,7 +1533,7 @@
         </is>
       </c>
       <c r="D8" s="14" t="n">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="E8" s="15" t="n">
         <v>0.09</v>
@@ -1603,12 +1603,12 @@
       </c>
       <c r="V8" s="13" t="inlineStr">
         <is>
-          <t>[V]</t>
+          <t>[V-RFQ]</t>
         </is>
       </c>
       <c r="W8" s="22" t="inlineStr">
         <is>
-          <t>Tianjin Kingnod BC-234BV $11-15, 5/caja — kingnodfurniture.en.made-in-china.com</t>
+          <t>RFQ 20-ago: Ningbo Metal Tech $10.50 (asiento madera)</t>
         </is>
       </c>
     </row>
@@ -1629,7 +1629,7 @@
         </is>
       </c>
       <c r="D9" s="14" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="E9" s="15" t="n">
         <v>0.09</v>
@@ -1699,12 +1699,12 @@
       </c>
       <c r="V9" s="13" t="inlineStr">
         <is>
-          <t>[V]</t>
+          <t>[V-RFQ]</t>
         </is>
       </c>
       <c r="W9" s="22" t="inlineStr">
         <is>
-          <t>Tianjin Kingnod $9.65-18.55</t>
+          <t>RFQ 20-ago: Ningbo $10.50 / Anji Shengtai $18.90 (18 años)</t>
         </is>
       </c>
     </row>
@@ -1821,7 +1821,7 @@
         </is>
       </c>
       <c r="D11" s="14" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="E11" s="15" t="n">
         <v>0.09</v>
@@ -1891,12 +1891,12 @@
       </c>
       <c r="V11" s="13" t="inlineStr">
         <is>
-          <t>[V]</t>
+          <t>[V-RFQ]</t>
         </is>
       </c>
       <c r="W11" s="22" t="inlineStr">
         <is>
-          <t>Langfang Bingwei $7.50-13.80 (Gold 2025 — pedir auditoría)</t>
+          <t>RFQ 20-ago: Ningbo Metal Tech $10.50</t>
         </is>
       </c>
     </row>
@@ -2013,7 +2013,7 @@
         </is>
       </c>
       <c r="D13" s="14" t="n">
-        <v>60</v>
+        <v>69</v>
       </c>
       <c r="E13" s="15" t="n">
         <v>0.2</v>
@@ -2055,10 +2055,10 @@
         <v/>
       </c>
       <c r="O13" s="19" t="n">
-        <v>3190</v>
+        <v>3390</v>
       </c>
       <c r="P13" s="19" t="n">
-        <v>3690</v>
+        <v>3890</v>
       </c>
       <c r="Q13" s="20">
         <f>O13-N13</f>
@@ -2083,12 +2083,12 @@
       </c>
       <c r="V13" s="13" t="inlineStr">
         <is>
-          <t>[V]</t>
+          <t>[V-RFQ]</t>
         </is>
       </c>
       <c r="W13" s="22" t="inlineStr">
         <is>
-          <t>Zhongshan Uptop $30-80 / Foshan Ron $39.90-139</t>
+          <t>RFQ 20-ago: Qingdao Green Forest $69 (redonda madera)</t>
         </is>
       </c>
     </row>
@@ -2397,7 +2397,7 @@
         </is>
       </c>
       <c r="D17" s="14" t="n">
-        <v>145</v>
+        <v>155</v>
       </c>
       <c r="E17" s="15" t="n">
         <v>0.45</v>
@@ -2439,10 +2439,10 @@
         <v/>
       </c>
       <c r="O17" s="19" t="n">
-        <v>7190</v>
+        <v>7590</v>
       </c>
       <c r="P17" s="19" t="n">
-        <v>8490</v>
+        <v>8890</v>
       </c>
       <c r="Q17" s="20">
         <f>O17-N17</f>
@@ -2467,12 +2467,12 @@
       </c>
       <c r="V17" s="13" t="inlineStr">
         <is>
-          <t>[V]</t>
+          <t>[V-RFQ]</t>
         </is>
       </c>
       <c r="W17" s="22" t="inlineStr">
         <is>
-          <t>Shanghai Miaolian PU lounge $143</t>
+          <t>RFQ 20-ago: Foshan Biaoguan $155.51 (reclinable madera)</t>
         </is>
       </c>
     </row>
@@ -2877,7 +2877,7 @@
         </is>
       </c>
       <c r="D22" s="14" t="n">
-        <v>42</v>
+        <v>16</v>
       </c>
       <c r="E22" s="15" t="n">
         <v>0.12</v>
@@ -2919,10 +2919,10 @@
         <v/>
       </c>
       <c r="O22" s="19" t="n">
-        <v>2490</v>
+        <v>1990</v>
       </c>
       <c r="P22" s="19" t="n">
-        <v>2990</v>
+        <v>2390</v>
       </c>
       <c r="Q22" s="20">
         <f>O22-N22</f>
@@ -2947,12 +2947,12 @@
       </c>
       <c r="V22" s="13" t="inlineStr">
         <is>
-          <t>[V]</t>
+          <t>[V-RFQ]</t>
         </is>
       </c>
       <c r="W22" s="22" t="inlineStr">
         <is>
-          <t>Foshan Zhongfayijia $39.99-49.99, 606/40'HQ — zhongfayijia.en.made-in-china.com</t>
+          <t>RFQ 20-ago: Foshan Qianmiao $13 (18 años OEM) / Anji Ka Bei Long $19</t>
         </is>
       </c>
     </row>
@@ -3357,7 +3357,7 @@
         </is>
       </c>
       <c r="D27" s="14" t="n">
-        <v>70</v>
+        <v>22</v>
       </c>
       <c r="E27" s="15" t="n">
         <v>0.16</v>
@@ -3399,10 +3399,10 @@
         <v/>
       </c>
       <c r="O27" s="19" t="n">
+        <v>2990</v>
+      </c>
+      <c r="P27" s="19" t="n">
         <v>3490</v>
-      </c>
-      <c r="P27" s="19" t="n">
-        <v>4190</v>
       </c>
       <c r="Q27" s="20">
         <f>O27-N27</f>
@@ -3427,12 +3427,12 @@
       </c>
       <c r="V27" s="13" t="inlineStr">
         <is>
-          <t>[V]</t>
+          <t>[V-RFQ]</t>
         </is>
       </c>
       <c r="W27" s="22" t="inlineStr">
         <is>
-          <t>Dongguan Z.MAX Sitzone T14 $63-75.60 / NOEL $57.70-86.60 (0.15 CBM=453/40')</t>
+          <t>RFQ 20-ago: Anji Wofeng $22 ejecutiva malla respaldo alto (verificar clase de pistón)</t>
         </is>
       </c>
     </row>
@@ -3741,7 +3741,7 @@
         </is>
       </c>
       <c r="D31" s="14" t="n">
-        <v>45</v>
+        <v>38</v>
       </c>
       <c r="E31" s="15" t="n">
         <v>0.14</v>
@@ -3811,12 +3811,12 @@
       </c>
       <c r="V31" s="13" t="inlineStr">
         <is>
-          <t>[V]</t>
+          <t>[V-RFQ]</t>
         </is>
       </c>
       <c r="W31" s="22" t="inlineStr">
         <is>
-          <t>BG Office Foshan $15-50</t>
+          <t>RFQ 20-ago: Hefei Maya $37.50/set escritorio ejecutivo madera</t>
         </is>
       </c>
     </row>
@@ -4413,7 +4413,7 @@
         </is>
       </c>
       <c r="D38" s="14" t="n">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="E38" s="15" t="n">
         <v>0.3</v>
@@ -4483,12 +4483,12 @@
       </c>
       <c r="V38" s="13" t="inlineStr">
         <is>
-          <t>[V]</t>
+          <t>[V-RFQ]</t>
         </is>
       </c>
       <c r="W38" s="22" t="inlineStr">
         <is>
-          <t>Linyi Gaotong aluminio fundido $62-70/set, garantía 3 años</t>
+          <t>RFQ 20-ago: Wuyi Sailing $69/set (14 años)</t>
         </is>
       </c>
     </row>
@@ -4605,7 +4605,7 @@
         </is>
       </c>
       <c r="D40" s="14" t="n">
-        <v>65</v>
+        <v>36</v>
       </c>
       <c r="E40" s="15" t="n">
         <v>0.3</v>
@@ -4675,12 +4675,12 @@
       </c>
       <c r="V40" s="13" t="inlineStr">
         <is>
-          <t>[V]</t>
+          <t>[V-RFQ]</t>
         </is>
       </c>
       <c r="W40" s="22" t="inlineStr">
         <is>
-          <t>Linyi Gaotong</t>
+          <t>RFQ 20-ago: Foshan Hongshi $35.84/set aluminio fundido</t>
         </is>
       </c>
     </row>

</xml_diff>